<commit_message>
Downgrade #2 (page refresh/back-forward) to Low priority
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/NcConnect_Bug_Tracker.xlsx
+++ b/NcConnect_Bug_Tracker.xlsx
@@ -46,6 +46,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001A7A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00CC6600"/>
       <sz val="10"/>
     </font>
@@ -53,12 +59,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00997A00"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001A7A4A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -89,6 +89,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E0F5EC"/>
+        <bgColor rgb="00E0F5EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF0DD"/>
         <bgColor rgb="00FFF0DD"/>
       </patternFill>
@@ -97,12 +103,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFCE0"/>
         <bgColor rgb="00FFFCE0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E0F5EC"/>
-        <bgColor rgb="00E0F5EC"/>
       </patternFill>
     </fill>
     <fill>
@@ -689,14 +689,14 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -724,7 +724,7 @@
           <t>Bug / UX</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -759,7 +759,7 @@
           <t>Bug / UX</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -794,7 +794,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -829,7 +829,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -864,7 +864,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -899,7 +899,7 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -934,7 +934,7 @@
           <t>Bug / UX</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -969,7 +969,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1004,7 +1004,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -1039,7 +1039,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -1074,7 +1074,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -1122,7 +1122,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1157,7 +1157,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1192,7 +1192,7 @@
           <t>Architecture</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>

<commit_message>
Move page refresh/back-forward to bottom of low priority section
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/NcConnect_Bug_Tracker.xlsx
+++ b/NcConnect_Bug_Tracker.xlsx
@@ -46,12 +46,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A7A4A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00CC6600"/>
       <sz val="10"/>
     </font>
@@ -59,6 +53,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00997A00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A7A4A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -89,12 +89,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0F5EC"/>
-        <bgColor rgb="00E0F5EC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF0DD"/>
         <bgColor rgb="00FFF0DD"/>
       </patternFill>
@@ -103,6 +97,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFCE0"/>
         <bgColor rgb="00FFFCE0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F5EC"/>
+        <bgColor rgb="00E0F5EC"/>
       </patternFill>
     </fill>
     <fill>
@@ -681,32 +681,32 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Page Refresh / Back-Forward Breaks Page Content</t>
+          <t>Summernote Save Workflow (Data Loss Risk)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Bug / UX</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Refreshing the page or using the browser’s back/forward buttons causes the page to break — only the blue title/header bar remains visible, with no content rendered below it and no buttons functional. This is distinct from the gray-out issue; the tab is still technically alive but completely unusable. Forces the user to open a new tab and re-navigate the full deep path, with the same context loss and productivity drain.</t>
+          <t>Saving in the Summernote editor while in code view silently discards all changes. The user must remember to exit code view first — there is no warning or safeguard. Results in lost work and rework.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Core Navigation</t>
+          <t>Code Editor</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Summernote Save Workflow (Data Loss Risk)</t>
+          <t>Product Save Workflow — Close &amp; Reopen Per Tab</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -724,7 +724,7 @@
           <t>Bug / UX</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -736,12 +736,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Saving in the Summernote editor while in code view silently discards all changes. The user must remember to exit code view first — there is no warning or safeguard. Results in lost work and rework.</t>
+          <t>Editing product details requires closing and reopening the product each time a different tab is modified. There is no way to save changes across multiple tabs in one session. Multi-field updates that should take a minute become a repetitive open-edit-close-reopen cycle.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Code Editor</t>
+          <t>Product Details</t>
         </is>
       </c>
     </row>
@@ -751,32 +751,32 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Product Save Workflow — Close &amp; Reopen Per Tab</t>
+          <t>FTP Definition Preview in Product Edit</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bug / UX</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Editing product details requires closing and reopening the product each time a different tab is modified. There is no way to save changes across multiple tabs in one session. Multi-field updates that should take a minute become a repetitive open-edit-close-reopen cycle.</t>
+          <t>No inline preview of the selected FTP definition when editing a product. To check the definition’s structure (and determine whether additional FTP tab fields need to be filled in), the user must leave the product, navigate to the FTP definitions area, locate the definition, review it, then deep-path navigate back. An inline preview on selection would eliminate this detour entirely.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Product Details</t>
+          <t>Product Details / FTP</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>FTP Definition Preview in Product Edit</t>
+          <t>PDF Preview Missing in Composition</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -794,7 +794,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -806,12 +806,12 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>No inline preview of the selected FTP definition when editing a product. To check the definition’s structure (and determine whether additional FTP tab fields need to be filled in), the user must leave the product, navigate to the FTP definitions area, locate the definition, review it, then deep-path navigate back. An inline preview on selection would eliminate this detour entirely.</t>
+          <t>The composition PDF view shows no preview, no filename, and no version info — just a download link with no context. Users must download the file to determine what version it is, making version comparison unnecessarily slow. Should display a preview (or at minimum filename + version label) and a clear download button.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Product Details / FTP</t>
+          <t>Composition</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>PDF Preview Missing in Composition</t>
+          <t>Code Editor Improvements</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -841,12 +841,12 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>The composition PDF view shows no preview, no filename, and no version info — just a download link with no context. Users must download the file to determine what version it is, making version comparison unnecessarily slow. Should display a preview (or at minimum filename + version label) and a clear download button.</t>
+          <t>The embedded editor is missing standard features expected in any code editing environment: no multi-cursor (Ctrl/Cmd-D), no reliable in-place save (must click out of the editor to trigger save), and no basic code formatting or linting. These gaps slow daily work across every template edit.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Composition</t>
+          <t>Code Editor</t>
         </is>
       </c>
     </row>
@@ -856,17 +856,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Code Editor Improvements</t>
+          <t>Server Capacity / Sample Creation Timing</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>The embedded editor is missing standard features expected in any code editing environment: no multi-cursor (Ctrl/Cmd-D), no reliable in-place save (must click out of the editor to trigger save), and no basic code formatting or linting. These gaps slow daily work across every template edit.</t>
+          <t>Sample creation runs on a fixed 5-minute interval rather than on-demand. Even a quick change requires waiting for the next cycle. This bottleneck may be a data server limitation. On-demand or near-immediate processing would tighten the edit-review loop significantly.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Code Editor</t>
+          <t>Server / Data</t>
         </is>
       </c>
     </row>
@@ -891,15 +891,15 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Server Capacity / Sample Creation Timing</t>
+          <t>Symbol / Special Character Limitations (Wingdings)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+          <t>Bug / UX</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -911,12 +911,12 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Sample creation runs on a fixed 5-minute interval rather than on-demand. Even a quick change requires waiting for the next cycle. This bottleneck may be a data server limitation. On-demand or near-immediate processing would tighten the edit-review loop significantly.</t>
+          <t>Special characters and symbols are restricted to the Wingdings font — likely due to Summernote, the print pipeline, or printer font constraints. Symbols that are clearly visible in the source Word document cannot be copy-pasted into the editor; instead, programmers must manually look up the corresponding Wingdings character code. A copy-paste workaround or a visual symbol picker mapping common symbols to their Wingdings equivalents would save significant time.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Server / Data</t>
+          <t>Code Editor / Summernote</t>
         </is>
       </c>
     </row>
@@ -926,15 +926,15 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Symbol / Special Character Limitations (Wingdings)</t>
+          <t>Error Transparency &amp; Observability</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bug / UX</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -946,12 +946,12 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Special characters and symbols are restricted to the Wingdings font — likely due to Summernote, the print pipeline, or printer font constraints. Symbols that are clearly visible in the source Word document cannot be copy-pasted into the editor; instead, programmers must manually look up the corresponding Wingdings character code. A copy-paste workaround or a visual symbol picker mapping common symbols to their Wingdings equivalents would save significant time.</t>
+          <t>Errors and failures across the platform are often silent or opaque. Suppressed files show no explanation, and error codes (when present) are not actionable. Users resort to manual investigation or guesswork. Clear, contextual error messages and accessible logs would reduce debugging time.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Code Editor / Summernote</t>
+          <t>Job Processing Screen</t>
         </is>
       </c>
     </row>
@@ -961,32 +961,32 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Error Transparency &amp; Observability</t>
+          <t>Dropdown Menus Overlap / Don’t Auto-Close</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Enhancement</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Errors and failures across the platform are often silent or opaque. Suppressed files show no explanation, and error codes (when present) are not actionable. Users resort to manual investigation or guesswork. Clear, contextual error messages and accessible logs would reduce debugging time.</t>
+          <t>Opening a new dropdown does not close the previously opened one, causing menus to overlap. Requires extra clicks to dismiss. Minor but persistent annoyance.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Job Processing Screen</t>
+          <t>Core UI</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Dropdown Menus Overlap / Don’t Auto-Close</t>
+          <t>‘X’ Button Misalignment on Company Filter</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1004,7 +1004,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Opening a new dropdown does not close the previously opened one, causing menus to overlap. Requires extra clicks to dismiss. Minor but persistent annoyance.</t>
+          <t>The close (‘X’) button on the company filter in the composition filter menu does not align with the mouse click target. Hitbox is offset from the visible button.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Core UI</t>
+          <t>Composition Filter</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>‘X’ Button Misalignment on Company Filter</t>
+          <t>Shift+Tab Navigation Broken on Dropdowns</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1039,7 +1039,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -1051,12 +1051,12 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>The close (‘X’) button on the company filter in the composition filter menu does not align with the mouse click target. Hitbox is offset from the visible button.</t>
+          <t>Tabbing forward through form fields works normally, but Shift+Tab (backwards) gets stuck on dropdown components. If a user overshoots a field, they cannot tab back to it and must use the mouse. Only affects reverse tab order.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Composition Filter</t>
+          <t>UI / Accessibility</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Shift+Tab Navigation Broken on Dropdowns</t>
+          <t>Page Refresh / Back-Forward Breaks Page Content</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1074,7 +1074,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -1086,12 +1086,12 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Tabbing forward through form fields works normally, but Shift+Tab (backwards) gets stuck on dropdown components. If a user overshoots a field, they cannot tab back to it and must use the mouse. Only affects reverse tab order.</t>
+          <t>Refreshing the page or using the browser’s back/forward buttons causes the page to break — only the blue title/header bar remains visible, with no content rendered below it and no buttons functional. This is distinct from the gray-out issue; the tab is still technically alive but completely unusable. Rare occurrence but unintuitive — standard browser actions shouldn’t break the page.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>UI / Accessibility</t>
+          <t>Core Navigation</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
           <t>Bug</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1157,7 +1157,7 @@
           <t>Enhancement</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1192,7 +1192,7 @@
           <t>Architecture</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>